<commit_message>
Double the gamma coefficient magnitude tiers (0.1/0.2/0.4 -> 0.2/0.4/0.8)
Scale the "Belegstaerke" evidence-strength legend in
fertigeabmparameter.xlsx (the gamma matrix cells reference these legend
cells by formula, so the whole 11-construct x 5-mode gamma matrix scales
with it) and propagate the resulting values into config.xml's gamma
params for all five alternatives.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scenarios/testszenario/fertigeabmparameter.xlsx
+++ b/scenarios/testszenario/fertigeabmparameter.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lel/IdeaProjects/matsim-example-project/scenarios/testszenario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90298544-51EB-A742-A58C-5B5EA2AF50C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF1D80F-A997-764C-9EFD-E6D6139B0BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15680" yWindow="680" windowWidth="18520" windowHeight="21460" xr2:uid="{D2D53BF3-C64E-0F44-8A9C-97E82D4EA947}"/>
+    <workbookView xWindow="12700" yWindow="680" windowWidth="21500" windowHeight="20480" xr2:uid="{D2D53BF3-C64E-0F44-8A9C-97E82D4EA947}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="46">
   <si>
     <t>Konstrukt</t>
   </si>
@@ -169,9 +172,6 @@
     <t>Kolarova et al. 2019; fuer alle drei AV-Modi generisch</t>
   </si>
   <si>
-    <t>Verteilung Wartezeit</t>
-  </si>
-  <si>
     <t>+++</t>
   </si>
   <si>
@@ -185,21 +185,6 @@
   </si>
   <si>
     <t>-</t>
-  </si>
-  <si>
-    <t>Vormodus: CA</t>
-  </si>
-  <si>
-    <t>Vormodus: PT</t>
-  </si>
-  <si>
-    <t>Vormodus: PAV</t>
-  </si>
-  <si>
-    <t>Vormodus: PSAV</t>
-  </si>
-  <si>
-    <t>Vormodus: SSAV</t>
   </si>
 </sst>
 </file>
@@ -334,7 +319,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -391,6 +376,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" quotePrefix="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -409,6 +397,32 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Lies_mich"/>
+      <sheetName val="Nach_Themen"/>
+      <sheetName val="Themen_Zusammenfassung"/>
+      <sheetName val="Erkenntnis_1_Spalte"/>
+      <sheetName val="Erkenntnisse"/>
+      <sheetName val="Original (unverändert)"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -749,14 +763,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B37D5553-6DC7-B641-A38D-8FE4527E225F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{B37D5553-6DC7-B641-A38D-8FE4527E225F}">
   <dimension ref="A1:N24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" ns3:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="56" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" ht="56" ns3:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -782,19 +796,19 @@
         <v>7</v>
       </c>
       <c r="K1" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="20">
+        <v>0.8</v>
+      </c>
+      <c r="M1" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="L1" s="20">
-        <v>0.4</v>
-      </c>
-      <c r="M1" s="21" t="s">
-        <v>43</v>
-      </c>
       <c r="N1" s="20">
-        <v>-0.4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="78" x14ac:dyDescent="0.2">
+        <v>-0.8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="78" ns3:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
@@ -809,33 +823,33 @@
       </c>
       <c r="E2" s="7">
         <f>$L$3</f>
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="F2" s="7">
         <f>$L$1</f>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="G2" s="7">
         <f>$L$2</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="H2" s="8" t="s">
         <v>10</v>
       </c>
       <c r="K2" s="21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L2" s="20">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="M2" s="21" t="s">
         <v>39</v>
       </c>
       <c r="N2" s="20">
-        <v>-0.2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ns3:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>21</v>
       </c>
@@ -847,36 +861,36 @@
       </c>
       <c r="D3" s="7">
         <f>$L$3</f>
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="E3" s="7">
         <f>$L$2</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="F3" s="6">
         <v>0</v>
       </c>
       <c r="G3" s="7">
         <f>$L$3</f>
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="H3" s="8" t="s">
         <v>14</v>
       </c>
       <c r="K3" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="L3" s="20">
+        <v>0.2</v>
+      </c>
+      <c r="M3" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="L3" s="20">
-        <v>0.1</v>
-      </c>
-      <c r="M3" s="21" t="s">
-        <v>46</v>
-      </c>
       <c r="N3" s="20">
-        <v>-0.1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ns3:dyDescent="0.2">
       <c r="A4" s="9" t="s">
         <v>22</v>
       </c>
@@ -885,28 +899,30 @@
       </c>
       <c r="C4" s="14">
         <f>$N$2</f>
-        <v>-0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="D4" s="10">
         <v>0</v>
       </c>
       <c r="E4" s="14">
         <f>$N$1</f>
-        <v>-0.4</v>
+        <v>-0.8</v>
       </c>
       <c r="F4" s="11">
         <f>$L$2</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="G4" s="11">
         <f>$L$1</f>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="H4" s="12" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" ht="52" x14ac:dyDescent="0.2">
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+    </row>
+    <row r="5" spans="1:14" ht="52" ns3:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>26</v>
       </c>
@@ -918,25 +934,25 @@
       </c>
       <c r="D5" s="14">
         <f>$N$2</f>
-        <v>-0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="E5" s="14">
         <f>$N$3</f>
-        <v>-0.1</v>
+        <v>-0.2</v>
       </c>
       <c r="F5" s="14">
         <f>$N$2</f>
-        <v>-0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="G5" s="14">
         <f>$N$2</f>
-        <v>-0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="H5" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="52" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" ht="52" ns3:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>11</v>
       </c>
@@ -951,21 +967,21 @@
       </c>
       <c r="E6" s="11">
         <f>$L$2</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="F6" s="11">
         <f>$L$2</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="G6" s="11">
         <f>$L$1</f>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="H6" s="12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="42" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" ht="42" ns3:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>13</v>
       </c>
@@ -980,20 +996,20 @@
       </c>
       <c r="E7" s="7">
         <f>$L$3</f>
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="F7" s="6">
         <v>0</v>
       </c>
       <c r="G7" s="7">
         <f>$L$3</f>
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" ns3:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>15</v>
       </c>
@@ -1005,24 +1021,24 @@
       </c>
       <c r="D8" s="11">
         <f>$L$1</f>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="E8" s="11">
         <f>$L$1</f>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="F8" s="10">
         <v>0</v>
       </c>
       <c r="G8" s="11">
         <f>$L$1</f>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="H8" s="12" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="28" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" ht="28" ns3:dyDescent="0.2">
       <c r="A9" s="9" t="s">
         <v>19</v>
       </c>
@@ -1031,27 +1047,27 @@
       </c>
       <c r="C9" s="11">
         <f>$L$1</f>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="D9" s="10">
         <v>0</v>
       </c>
       <c r="E9" s="11">
         <f>$L$2</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="F9" s="10">
         <v>0</v>
       </c>
       <c r="G9" s="11">
         <f>$L$1</f>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="H9" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="65" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" ht="65" ns3:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>17</v>
       </c>
@@ -1066,20 +1082,20 @@
       </c>
       <c r="E10" s="13">
         <f>$N$2</f>
-        <v>-0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="F10" s="6">
         <v>0</v>
       </c>
       <c r="G10" s="13">
         <f>$N$2</f>
-        <v>-0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="65" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" ht="65" ns3:dyDescent="0.2">
       <c r="A11" s="9" t="s">
         <v>24</v>
       </c>
@@ -1094,20 +1110,20 @@
       </c>
       <c r="E11" s="11">
         <f>$L$2</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="F11" s="10">
         <v>0</v>
       </c>
       <c r="G11" s="11">
         <f>$L$1</f>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="H11" s="12" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="28" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" ht="28" ns3:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>23</v>
       </c>
@@ -1122,21 +1138,21 @@
       </c>
       <c r="E12" s="7">
         <f>$L$2</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="F12" s="7">
         <f>$L$1</f>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="G12" s="7">
         <f>$L$1</f>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" ns3:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>28</v>
       </c>
@@ -1160,7 +1176,7 @@
       </c>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" ns3:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>30</v>
       </c>
@@ -1184,7 +1200,7 @@
       </c>
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" ns3:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>31</v>
       </c>
@@ -1208,7 +1224,7 @@
       </c>
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:14" ht="78" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" ht="78" ns3:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>32</v>
       </c>
@@ -1216,7 +1232,8 @@
         <v>33</v>
       </c>
       <c r="C16" s="17">
-        <v>-0.105</v>
+        <f>[1]Themen_Zusammenfassung!$E$4</f>
+        <v>0</v>
       </c>
       <c r="D16" s="17">
         <v>-5.7700000000000001E-2</v>
@@ -1234,7 +1251,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" ns3:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>35</v>
       </c>
@@ -1258,7 +1275,7 @@
       </c>
       <c r="H17" s="16"/>
     </row>
-    <row r="18" spans="1:8" ht="65" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" ht="65" ns3:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>38</v>
       </c>
@@ -1284,132 +1301,57 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="D19" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="E19" s="17">
-        <v>0.29799999999999999</v>
-      </c>
-      <c r="F19" s="17">
-        <v>0.29799999999999999</v>
-      </c>
-      <c r="G19" s="17">
-        <v>0.29799999999999999</v>
-      </c>
+    <row r="19" spans="1:8" ns3:dyDescent="0.2">
+      <c r="A19" s="22"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
       <c r="H19" s="16"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="C20" s="23">
-        <v>1.73</v>
-      </c>
-      <c r="D20" s="23">
-        <v>0</v>
-      </c>
-      <c r="E20" s="23">
-        <v>0.95</v>
-      </c>
-      <c r="F20" s="23">
-        <v>0.63</v>
-      </c>
-      <c r="G20" s="23">
-        <v>0.95</v>
-      </c>
+    <row r="20" spans="1:8" ns3:dyDescent="0.2">
+      <c r="C20" s="23"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
       <c r="H20" s="20"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="C21" s="23">
-        <v>0</v>
-      </c>
-      <c r="D21" s="23">
-        <v>0.85</v>
-      </c>
-      <c r="E21" s="23">
-        <v>0</v>
-      </c>
-      <c r="F21" s="23">
-        <v>0.95</v>
-      </c>
-      <c r="G21" s="23">
-        <v>0.45</v>
-      </c>
+    <row r="21" spans="1:8" ns3:dyDescent="0.2">
+      <c r="A21" s="22"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
       <c r="H21" s="20"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="22" t="s">
-        <v>49</v>
-      </c>
-      <c r="C22" s="23">
-        <v>0.45</v>
-      </c>
-      <c r="D22" s="23">
-        <v>0</v>
-      </c>
-      <c r="E22" s="23">
-        <v>1.73</v>
-      </c>
-      <c r="F22" s="23">
-        <v>0.45</v>
-      </c>
-      <c r="G22" s="23">
-        <v>0.45</v>
-      </c>
+    <row r="22" spans="1:8" ns3:dyDescent="0.2">
+      <c r="A22" s="22"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
       <c r="H22" s="16"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="22" t="s">
-        <v>50</v>
-      </c>
-      <c r="C23" s="23">
-        <v>0</v>
-      </c>
-      <c r="D23" s="23">
-        <v>0.45</v>
-      </c>
-      <c r="E23" s="23">
-        <v>0.45</v>
-      </c>
-      <c r="F23" s="23">
-        <v>1.73</v>
-      </c>
-      <c r="G23" s="23">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="C24" s="23">
-        <v>0.45</v>
-      </c>
-      <c r="D24" s="23">
-        <v>0</v>
-      </c>
-      <c r="E24" s="23">
-        <v>0.45</v>
-      </c>
-      <c r="F24" s="23">
-        <v>0.95</v>
-      </c>
-      <c r="G24" s="23">
-        <v>1.73</v>
-      </c>
+    <row r="23" spans="1:8" ns3:dyDescent="0.2">
+      <c r="A23" s="22"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
+    </row>
+    <row r="24" spans="1:8" ns3:dyDescent="0.2">
+      <c r="A24" s="22"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Set all mode ASCs to 0 and revert gamma tiers back to 0.1/0.2/0.4
ascSd values are left untouched. The gamma magnitude legend in
fertigeabmparameter.xlsx reverts to its pre-doubling values
(0.1/0.2/0.4), undoing fd2d147; config.xml's five gamma params are
updated to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scenarios/testszenario/fertigeabmparameter.xlsx
+++ b/scenarios/testszenario/fertigeabmparameter.xlsx
@@ -799,13 +799,13 @@
         <v>41</v>
       </c>
       <c r="L1" s="20">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="M1" s="21" t="s">
         <v>42</v>
       </c>
       <c r="N1" s="20">
-        <v>-0.8</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="78" ns3:dyDescent="0.2">
@@ -823,15 +823,15 @@
       </c>
       <c r="E2" s="7">
         <f>$L$3</f>
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="F2" s="7">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="G2" s="7">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="H2" s="8" t="s">
         <v>10</v>
@@ -840,13 +840,13 @@
         <v>43</v>
       </c>
       <c r="L2" s="20">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="M2" s="21" t="s">
         <v>39</v>
       </c>
       <c r="N2" s="20">
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="3" spans="1:14" ns3:dyDescent="0.2">
@@ -861,18 +861,18 @@
       </c>
       <c r="D3" s="7">
         <f>$L$3</f>
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="E3" s="7">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F3" s="6">
         <v>0</v>
       </c>
       <c r="G3" s="7">
         <f>$L$3</f>
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="H3" s="8" t="s">
         <v>14</v>
@@ -881,13 +881,13 @@
         <v>44</v>
       </c>
       <c r="L3" s="20">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="M3" s="21" t="s">
         <v>45</v>
       </c>
       <c r="N3" s="20">
-        <v>-0.2</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="4" spans="1:14" ns3:dyDescent="0.2">
@@ -899,22 +899,22 @@
       </c>
       <c r="C4" s="14">
         <f>$N$2</f>
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="D4" s="10">
         <v>0</v>
       </c>
       <c r="E4" s="14">
         <f>$N$1</f>
-        <v>-0.8</v>
+        <v>-0.4</v>
       </c>
       <c r="F4" s="11">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="G4" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H4" s="12" t="s">
         <v>16</v>
@@ -934,19 +934,19 @@
       </c>
       <c r="D5" s="14">
         <f>$N$2</f>
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="E5" s="14">
         <f>$N$3</f>
-        <v>-0.2</v>
+        <v>-0.1</v>
       </c>
       <c r="F5" s="14">
         <f>$N$2</f>
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="G5" s="14">
         <f>$N$2</f>
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="H5" s="12" t="s">
         <v>27</v>
@@ -967,15 +967,15 @@
       </c>
       <c r="E6" s="11">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F6" s="11">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="G6" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H6" s="12" t="s">
         <v>12</v>
@@ -996,14 +996,14 @@
       </c>
       <c r="E7" s="7">
         <f>$L$3</f>
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="F7" s="6">
         <v>0</v>
       </c>
       <c r="G7" s="7">
         <f>$L$3</f>
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>14</v>
@@ -1021,18 +1021,18 @@
       </c>
       <c r="D8" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="E8" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="F8" s="10">
         <v>0</v>
       </c>
       <c r="G8" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H8" s="12" t="s">
         <v>16</v>
@@ -1047,21 +1047,21 @@
       </c>
       <c r="C9" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="D9" s="10">
         <v>0</v>
       </c>
       <c r="E9" s="11">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F9" s="10">
         <v>0</v>
       </c>
       <c r="G9" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H9" s="12" t="s">
         <v>20</v>
@@ -1082,14 +1082,14 @@
       </c>
       <c r="E10" s="13">
         <f>$N$2</f>
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="F10" s="6">
         <v>0</v>
       </c>
       <c r="G10" s="13">
         <f>$N$2</f>
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>18</v>
@@ -1110,14 +1110,14 @@
       </c>
       <c r="E11" s="11">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F11" s="10">
         <v>0</v>
       </c>
       <c r="G11" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H11" s="12" t="s">
         <v>25</v>
@@ -1138,15 +1138,15 @@
       </c>
       <c r="E12" s="7">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F12" s="7">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="G12" s="7">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
Halve gamma coefficient tiers back to 0.4/0.2/0.1, set lastIteration back to 30
Reverts the gamma doubling from 03d6e3b (config.xml gamma/asc/ascNull
restored to the pre-doubling 69a22ee values, fertigeabmparameter.xlsx
Belegstaerke legend cells L1-3/N1-3 halved back to 0.4/0.2/0.1 with all
32 referencing formula cells' cached values updated to match) and
raises lastIteration back to 30 for the next full run now that the
DRT fleet-size shrinking is disabled.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYCx7ZofZADZz13NFvpkrR
</commit_message>
<xml_diff>
--- a/scenarios/testszenario/fertigeabmparameter.xlsx
+++ b/scenarios/testszenario/fertigeabmparameter.xlsx
@@ -799,13 +799,13 @@
         <v>41</v>
       </c>
       <c r="L1" s="20">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="M1" s="21" t="s">
         <v>42</v>
       </c>
       <c r="N1" s="20">
-        <v>-0.8</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="78" ns3:dyDescent="0.2">
@@ -823,15 +823,15 @@
       </c>
       <c r="E2" s="7">
         <f>$L$3</f>
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="F2" s="7">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="G2" s="7">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="H2" s="8" t="s">
         <v>10</v>
@@ -840,13 +840,13 @@
         <v>43</v>
       </c>
       <c r="L2" s="20">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="M2" s="21" t="s">
         <v>39</v>
       </c>
       <c r="N2" s="20">
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="3" spans="1:14" ns3:dyDescent="0.2">
@@ -861,18 +861,18 @@
       </c>
       <c r="D3" s="7">
         <f>$L$3</f>
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="E3" s="7">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F3" s="6">
         <v>0</v>
       </c>
       <c r="G3" s="7">
         <f>$L$3</f>
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="H3" s="8" t="s">
         <v>14</v>
@@ -881,13 +881,13 @@
         <v>44</v>
       </c>
       <c r="L3" s="20">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="M3" s="21" t="s">
         <v>45</v>
       </c>
       <c r="N3" s="20">
-        <v>-0.2</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="4" spans="1:14" ns3:dyDescent="0.2">
@@ -899,22 +899,22 @@
       </c>
       <c r="C4" s="14">
         <f>$N$2</f>
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="D4" s="10">
         <v>0</v>
       </c>
       <c r="E4" s="14">
         <f>$N$1</f>
-        <v>-0.8</v>
+        <v>-0.4</v>
       </c>
       <c r="F4" s="11">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="G4" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H4" s="12" t="s">
         <v>16</v>
@@ -934,19 +934,19 @@
       </c>
       <c r="D5" s="14">
         <f>$N$2</f>
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="E5" s="14">
         <f>$N$3</f>
-        <v>-0.2</v>
+        <v>-0.1</v>
       </c>
       <c r="F5" s="14">
         <f>$N$2</f>
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="G5" s="14">
         <f>$N$2</f>
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="H5" s="12" t="s">
         <v>27</v>
@@ -967,15 +967,15 @@
       </c>
       <c r="E6" s="11">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F6" s="11">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="G6" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H6" s="12" t="s">
         <v>12</v>
@@ -996,14 +996,14 @@
       </c>
       <c r="E7" s="7">
         <f>$L$3</f>
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="F7" s="6">
         <v>0</v>
       </c>
       <c r="G7" s="7">
         <f>$L$3</f>
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>14</v>
@@ -1021,18 +1021,18 @@
       </c>
       <c r="D8" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="E8" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="F8" s="10">
         <v>0</v>
       </c>
       <c r="G8" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H8" s="12" t="s">
         <v>16</v>
@@ -1047,21 +1047,21 @@
       </c>
       <c r="C9" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="D9" s="10">
         <v>0</v>
       </c>
       <c r="E9" s="11">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F9" s="10">
         <v>0</v>
       </c>
       <c r="G9" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H9" s="12" t="s">
         <v>20</v>
@@ -1082,14 +1082,14 @@
       </c>
       <c r="E10" s="13">
         <f>$N$2</f>
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="F10" s="6">
         <v>0</v>
       </c>
       <c r="G10" s="13">
         <f>$N$2</f>
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>18</v>
@@ -1110,14 +1110,14 @@
       </c>
       <c r="E11" s="11">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F11" s="10">
         <v>0</v>
       </c>
       <c r="G11" s="11">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H11" s="12" t="s">
         <v>25</v>
@@ -1138,15 +1138,15 @@
       </c>
       <c r="E12" s="7">
         <f>$L$2</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F12" s="7">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="G12" s="7">
         <f>$L$1</f>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>20</v>

</xml_diff>